<commit_message>
test(core): round-trip test (xlsx ↔ Network ↔ dbc for all valid fixtures) + deepEqualNetwork
deepEqualNetwork normalizes two known DBC asymmetries:
  - node.address is dropped by parseDbc (BU_ has no address slot)
  - signal.valueTable reference name may differ after a DBC round-trip
    because parseDbc binds by signal name; the valueTables list itself
    is deduped by entry set for comparison.

This keeps the round-trip test stable while exposing any future
field-level asymmetry as a diff.
</commit_message>
<xml_diff>
--- a/samples/valid/powertrain-typical/input.xlsx
+++ b/samples/valid/powertrain-typical/input.xlsx
@@ -152,16 +152,16 @@
     <t>Gear</t>
   </si>
   <si>
+    <t>OilTemp</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>degC</t>
+  </si>
+  <si>
     <t>GearTable</t>
-  </si>
-  <si>
-    <t>OilTemp</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>degC</t>
   </si>
   <si>
     <t>Raw Value</t>
@@ -949,7 +949,7 @@
         <v>4</v>
       </c>
       <c r="O4" t="s">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="P4" t="s">
         <v>3</v>
@@ -972,7 +972,7 @@
         <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
         <v>4</v>
@@ -993,7 +993,7 @@
         <v>39</v>
       </c>
       <c r="I5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -1008,7 +1008,7 @@
         <v>215</v>
       </c>
       <c r="N5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O5" t="s">
         <v>4</v>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -1080,7 +1080,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1091,7 +1091,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1102,7 +1102,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -1113,7 +1113,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B5">
         <v>3</v>

</xml_diff>